<commit_message>
Final excel sheet documentation
</commit_message>
<xml_diff>
--- a/Excel files/Defect_Tracker Template InfySpringboard.xlsx
+++ b/Excel files/Defect_Tracker Template InfySpringboard.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30606"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://infosystechnologies-my.sharepoint.com/personal/kamaljeet_kaur01_ad_infosys_com1/Documents/Infosys/CC/Events/Oct 2021 - Mar 2022/CC2.0/Internship/Jan-Apr 2022/Artifacts/internship/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="167" documentId="13_ncr:101_{A9B59A9A-789B-4A89-A90D-BB9A1B756E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{237CA605-A4BD-45B3-9AC6-47EAC7EDD262}"/>
+  <xr:revisionPtr revIDLastSave="228" documentId="13_ncr:101_{A9B59A9A-789B-4A89-A90D-BB9A1B756E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD4C0331-6342-41D5-BEA3-33354F81C205}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Defects" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="51">
   <si>
     <t>Sl No</t>
   </si>
@@ -159,7 +159,25 @@
     <t>Added CRITICAL RULE to prompt and python parsing logic to auto-generate INC-XXXX.md tickets.</t>
   </si>
   <si>
-    <t>.</t>
+    <t>Frontend API requests using incorrect backend URL.</t>
+  </si>
+  <si>
+    <t>Sprint 4</t>
+  </si>
+  <si>
+    <t>Configured the frontend API URL for backend connectivity.</t>
+  </si>
+  <si>
+    <t>Frontend routes failing on direct navigation or refresh.</t>
+  </si>
+  <si>
+    <t>Configure vercel writing in verel.json</t>
+  </si>
+  <si>
+    <t>Production API connectivity requires verification after deployment</t>
+  </si>
+  <si>
+    <t>Configured Render startup command and frontend environment settings</t>
   </si>
   <si>
     <t>User Interface</t>
@@ -178,7 +196,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -187,14 +205,6 @@
       <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -236,32 +246,46 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="12"/>
-      <color rgb="FF1F2328"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="-Apple-System"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
-      <color rgb="FFD1D7E0"/>
-      <name val="-Apple-System"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="-Apple-System"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFD1D7E0"/>
+      <color theme="1"/>
       <name val="Ui-Monospace"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Ui-Monospace"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -278,7 +302,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -302,15 +326,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -322,19 +337,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -353,83 +355,72 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -735,481 +726,558 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr defaultColWidth="17.5703125" defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="43.7109375" style="4" customWidth="1"/>
-    <col min="5" max="5" width="16" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="98.7109375" style="4" customWidth="1"/>
-    <col min="9" max="10" width="21.85546875" style="4" customWidth="1"/>
-    <col min="11" max="11" width="16.85546875" style="4" customWidth="1"/>
-    <col min="12" max="16384" width="17.5703125" style="4"/>
+    <col min="1" max="1" width="6.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="95.28515625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="16" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="98.7109375" style="3" customWidth="1"/>
+    <col min="9" max="10" width="21.85546875" style="3" customWidth="1"/>
+    <col min="11" max="11" width="16.85546875" style="3" customWidth="1"/>
+    <col min="12" max="16384" width="17.5703125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="31.5">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" s="1" customFormat="1" ht="32.25">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="8" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="64.5">
-      <c r="A2" s="3">
+      <c r="L1" s="20"/>
+    </row>
+    <row r="2" spans="1:12" ht="16.5">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="8">
+      <c r="B2" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="10">
         <v>46268</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="3" t="s">
+      <c r="F2" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="9" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="64.5">
-      <c r="A3" s="3">
+      <c r="L2" s="21"/>
+    </row>
+    <row r="3" spans="1:12" ht="16.5">
+      <c r="A3" s="9">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="8">
+      <c r="B3" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="10">
         <v>46268</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" s="9" t="s">
+      <c r="F3" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="9" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" ht="48.75">
-      <c r="A4" s="3">
+      <c r="L3" s="21"/>
+    </row>
+    <row r="4" spans="1:12" ht="32.25">
+      <c r="A4" s="9">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="3" t="s">
+      <c r="F4" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="9" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="32.25">
-      <c r="A5" s="3">
+      <c r="L4" s="21"/>
+    </row>
+    <row r="5" spans="1:12" ht="16.5">
+      <c r="A5" s="9">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="12" t="s">
+      <c r="B5" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="3" t="s">
+      <c r="F5" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="9" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="32.25">
-      <c r="A6" s="3">
+      <c r="L5" s="21"/>
+    </row>
+    <row r="6" spans="1:12" ht="16.5">
+      <c r="A6" s="9">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="3" t="s">
+      <c r="B6" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="3" t="s">
+      <c r="F6" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="H6" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="K6" s="9" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" ht="15.75">
-      <c r="A7" s="16">
+      <c r="L6" s="21"/>
+    </row>
+    <row r="7" spans="1:12" ht="15.75">
+      <c r="A7" s="14">
         <v>6</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="14" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="16" t="s">
+      <c r="F7" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="21" t="s">
+      <c r="H7" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="I7" s="17" t="s">
+      <c r="I7" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="J7" s="17" t="s">
+      <c r="J7" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="18" t="s">
+      <c r="K7" s="14" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="17">
+      <c r="L7" s="21"/>
+    </row>
+    <row r="8" spans="1:12" ht="15.75">
+      <c r="A8" s="14">
         <v>7</v>
       </c>
-      <c r="B8" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="17" t="s">
+      <c r="B8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="19" t="s">
+      <c r="F8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="23" t="s">
+      <c r="H8" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="I8" s="20" t="s">
+      <c r="I8" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="J8" s="17" t="s">
+      <c r="J8" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K8" s="17" t="s">
+      <c r="K8" s="14" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="15.75">
-      <c r="A9" s="16">
+      <c r="L8" s="21"/>
+    </row>
+    <row r="9" spans="1:12" ht="15.75">
+      <c r="A9" s="14">
         <v>8</v>
       </c>
-      <c r="B9" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="16" t="s">
+      <c r="B9" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="22" t="s">
+      <c r="F9" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="27" t="s">
+      <c r="H9" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="I9" s="20" t="s">
+      <c r="I9" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="J9" s="17" t="s">
+      <c r="J9" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="K9" s="18" t="s">
+      <c r="K9" s="14" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" ht="15.75">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="6"/>
-    </row>
-    <row r="11" spans="1:11" ht="15.75">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="11" t="s">
+      <c r="L9" s="21"/>
+    </row>
+    <row r="10" spans="1:12" ht="16.5">
+      <c r="A10" s="9">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="17">
+        <v>46063</v>
+      </c>
+      <c r="D10" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-    </row>
-    <row r="12" spans="1:11" ht="15.75">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="6"/>
-    </row>
-    <row r="13" spans="1:11" ht="15.75">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-    </row>
-    <row r="14" spans="1:11" ht="15.75">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="6"/>
-    </row>
-    <row r="15" spans="1:11" ht="15.75">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-    </row>
-    <row r="16" spans="1:11" ht="15.75">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="6"/>
+      <c r="E10" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I10" s="17">
+        <v>46063</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="L10" s="21"/>
+    </row>
+    <row r="11" spans="1:12" ht="16.5">
+      <c r="A11" s="9">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="17">
+        <v>46091</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="I11" s="17">
+        <v>46091</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="L11" s="21"/>
+    </row>
+    <row r="12" spans="1:12" ht="16.5">
+      <c r="A12" s="9">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="17">
+        <v>46213</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H12" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="I12" s="17">
+        <v>46213</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="L12" s="21"/>
+    </row>
+    <row r="13" spans="1:12" ht="15.75">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="21"/>
+    </row>
+    <row r="14" spans="1:12" ht="15.75">
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="24"/>
+    </row>
+    <row r="15" spans="1:12" ht="15.75">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+    </row>
+    <row r="16" spans="1:12" ht="15.75">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="5"/>
     </row>
     <row r="17" spans="1:11" ht="15.75">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="6"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="5"/>
     </row>
     <row r="18" spans="1:11" ht="15.75">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="6"/>
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="5"/>
     </row>
     <row r="19" spans="1:11" ht="15.75">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
     </row>
     <row r="20" spans="1:11" ht="15.75">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="6"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1243,22 +1311,22 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="7" t="s">
-        <v>44</v>
+      <c r="A5" s="6" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1274,15 +1342,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F50FC49184C87E449886FB52439922C9" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f85b7e58c3d8889ba0673e7b34a193a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b67b99c0-208c-4860-83e0-51466af787c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d43477c1ade21a66d9a75ba2d5aa042" ns2:_="">
     <xsd:import namespace="b67b99c0-208c-4860-83e0-51466af787c4"/>
@@ -1414,14 +1473,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}"/>
 </file>
</xml_diff>